<commit_message>
run models and update species traits for new species from new cities
</commit_message>
<xml_diff>
--- a/data/lepidoptera_trait_data/lepidoptera_trait_data/SpeciesListForTraits.xlsx
+++ b/data/lepidoptera_trait_data/lepidoptera_trait_data/SpeciesListForTraits.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jensj\Documents\R\urban_park_community_science_project\data\lepidoptera_trait_data\lepidoptera_trait_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1FE8D32-5B7B-448D-91C4-92806129FC97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39ED4413-2097-4DF8-BCBA-2CA1B620D333}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="899" uniqueCount="485">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="900" uniqueCount="487">
   <si>
     <t>aveWingspan</t>
   </si>
@@ -1491,6 +1491,12 @@
   </si>
   <si>
     <t>Polites coras</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>wingspan value is the average from BAMONA</t>
   </si>
 </sst>
 </file>
@@ -2359,7 +2365,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA329"/>
+  <dimension ref="A1:AB329"/>
   <sheetFormatPr defaultColWidth="10.83203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26.83203125" style="1" customWidth="1"/>
@@ -2373,7 +2379,7 @@
     <col min="28" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>354</v>
       </c>
@@ -2455,8 +2461,11 @@
       <c r="AA1" t="s">
         <v>454</v>
       </c>
-    </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB1" s="1" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>20</v>
       </c>
@@ -2535,7 +2544,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -2612,7 +2621,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>294</v>
       </c>
@@ -2691,7 +2700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>295</v>
       </c>
@@ -2774,7 +2783,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>22</v>
       </c>
@@ -2853,7 +2862,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>23</v>
       </c>
@@ -2930,7 +2939,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -3007,7 +3016,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>309</v>
       </c>
@@ -3086,7 +3095,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>310</v>
       </c>
@@ -3165,7 +3174,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>311</v>
       </c>
@@ -3244,7 +3253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -3321,7 +3330,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -3398,7 +3407,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -3475,7 +3484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -3552,7 +3561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>296</v>
       </c>
@@ -19233,7 +19242,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
         <v>203</v>
       </c>
@@ -19244,8 +19253,8 @@
       <c r="D225"/>
       <c r="E225"/>
       <c r="F225"/>
-      <c r="G225" t="s">
-        <v>321</v>
+      <c r="G225" s="3">
+        <v>8.5</v>
       </c>
       <c r="H225">
         <v>0</v>
@@ -19307,8 +19316,11 @@
       <c r="AA225" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="226" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AB225" s="1" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="226" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
         <v>204</v>
       </c>
@@ -19383,7 +19395,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="227" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
         <v>205</v>
       </c>
@@ -19458,7 +19470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
         <v>206</v>
       </c>
@@ -19533,7 +19545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
         <v>207</v>
       </c>
@@ -19608,7 +19620,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="230" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
         <v>208</v>
       </c>
@@ -19683,7 +19695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="231" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A231" s="3"/>
       <c r="B231" s="3" t="s">
         <v>478</v>
@@ -19734,7 +19746,7 @@
       </c>
       <c r="AA231" s="3"/>
     </row>
-    <row r="232" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
         <v>318</v>
       </c>
@@ -19813,7 +19825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="233" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
         <v>209</v>
       </c>
@@ -19888,7 +19900,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="234" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
         <v>210</v>
       </c>
@@ -19963,7 +19975,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="235" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
         <v>211</v>
       </c>
@@ -20038,7 +20050,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="236" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
         <v>212</v>
       </c>
@@ -20113,7 +20125,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="237" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
         <v>213</v>
       </c>
@@ -20188,7 +20200,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="238" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
         <v>214</v>
       </c>
@@ -20263,7 +20275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="239" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
         <v>319</v>
       </c>
@@ -20342,7 +20354,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="240" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A240" t="s">
         <v>300</v>
       </c>

</xml_diff>

<commit_message>
update species traits for southeast (didn't add florida cities yet)
</commit_message>
<xml_diff>
--- a/data/lepidoptera_trait_data/lepidoptera_trait_data/SpeciesListForTraits.xlsx
+++ b/data/lepidoptera_trait_data/lepidoptera_trait_data/SpeciesListForTraits.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jensj\Documents\R\urban_park_community_science_project\data\lepidoptera_trait_data\lepidoptera_trait_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CA3A4CB-E732-441A-9E7E-48558E2AEDCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26DFAB9F-CF56-4491-9C71-3673640F61DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="493">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="495">
   <si>
     <t>aveWingspan</t>
   </si>
@@ -1515,6 +1515,12 @@
   </si>
   <si>
     <t>Oarisma aurantiaca</t>
+  </si>
+  <si>
+    <t>Mastor celia</t>
+  </si>
+  <si>
+    <t>Polites egeremet</t>
   </si>
 </sst>
 </file>
@@ -2390,7 +2396,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB335"/>
+  <dimension ref="A1:AB336"/>
   <sheetFormatPr defaultColWidth="10.83203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26.83203125" style="1" customWidth="1"/>
@@ -3282,7 +3288,9 @@
       <c r="A12" t="s">
         <v>25</v>
       </c>
-      <c r="B12"/>
+      <c r="B12" s="3" t="s">
+        <v>493</v>
+      </c>
       <c r="C12" t="s">
         <v>25</v>
       </c>
@@ -27452,7 +27460,7 @@
         <v>292</v>
       </c>
       <c r="B334" s="3" t="s">
-        <v>489</v>
+        <v>494</v>
       </c>
       <c r="C334" t="s">
         <v>451</v>
@@ -27526,76 +27534,153 @@
     </row>
     <row r="335" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A335" t="s">
-        <v>293</v>
-      </c>
-      <c r="B335" t="s">
-        <v>293</v>
-      </c>
-      <c r="C335"/>
+        <v>292</v>
+      </c>
+      <c r="B335" s="3" t="s">
+        <v>489</v>
+      </c>
+      <c r="C335" t="s">
+        <v>451</v>
+      </c>
       <c r="D335"/>
       <c r="E335"/>
       <c r="F335"/>
       <c r="G335">
+        <v>2.9</v>
+      </c>
+      <c r="H335">
+        <v>1</v>
+      </c>
+      <c r="I335">
+        <v>0</v>
+      </c>
+      <c r="J335">
+        <v>0</v>
+      </c>
+      <c r="K335">
+        <v>1</v>
+      </c>
+      <c r="L335">
+        <v>1</v>
+      </c>
+      <c r="M335">
+        <v>1</v>
+      </c>
+      <c r="N335">
+        <v>0</v>
+      </c>
+      <c r="O335">
+        <v>0</v>
+      </c>
+      <c r="P335">
+        <v>0</v>
+      </c>
+      <c r="Q335">
+        <v>0</v>
+      </c>
+      <c r="R335">
+        <v>0</v>
+      </c>
+      <c r="S335">
+        <v>0</v>
+      </c>
+      <c r="T335">
+        <v>0</v>
+      </c>
+      <c r="U335">
+        <v>0</v>
+      </c>
+      <c r="V335">
+        <v>0</v>
+      </c>
+      <c r="W335">
+        <v>1</v>
+      </c>
+      <c r="X335">
+        <v>1</v>
+      </c>
+      <c r="Y335">
+        <v>4</v>
+      </c>
+      <c r="Z335">
+        <v>2</v>
+      </c>
+      <c r="AA335" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="336" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A336" t="s">
+        <v>293</v>
+      </c>
+      <c r="B336" t="s">
+        <v>293</v>
+      </c>
+      <c r="C336"/>
+      <c r="D336"/>
+      <c r="E336"/>
+      <c r="F336"/>
+      <c r="G336">
         <v>5.2673611109999996</v>
       </c>
-      <c r="H335">
-        <v>1</v>
-      </c>
-      <c r="I335">
-        <v>0</v>
-      </c>
-      <c r="J335">
-        <v>0</v>
-      </c>
-      <c r="K335">
-        <v>0</v>
-      </c>
-      <c r="L335">
-        <v>0</v>
-      </c>
-      <c r="M335">
-        <v>0</v>
-      </c>
-      <c r="N335">
-        <v>1</v>
-      </c>
-      <c r="O335">
-        <v>0</v>
-      </c>
-      <c r="P335">
-        <v>0</v>
-      </c>
-      <c r="Q335">
-        <v>1</v>
-      </c>
-      <c r="R335">
-        <v>0</v>
-      </c>
-      <c r="S335">
-        <v>0</v>
-      </c>
-      <c r="T335">
-        <v>0</v>
-      </c>
-      <c r="U335">
-        <v>0</v>
-      </c>
-      <c r="V335">
-        <v>0</v>
-      </c>
-      <c r="W335">
-        <v>0</v>
-      </c>
-      <c r="X335">
-        <v>0</v>
-      </c>
-      <c r="Y335">
+      <c r="H336">
+        <v>1</v>
+      </c>
+      <c r="I336">
+        <v>0</v>
+      </c>
+      <c r="J336">
+        <v>0</v>
+      </c>
+      <c r="K336">
+        <v>0</v>
+      </c>
+      <c r="L336">
+        <v>0</v>
+      </c>
+      <c r="M336">
+        <v>0</v>
+      </c>
+      <c r="N336">
+        <v>1</v>
+      </c>
+      <c r="O336">
+        <v>0</v>
+      </c>
+      <c r="P336">
+        <v>0</v>
+      </c>
+      <c r="Q336">
+        <v>1</v>
+      </c>
+      <c r="R336">
+        <v>0</v>
+      </c>
+      <c r="S336">
+        <v>0</v>
+      </c>
+      <c r="T336">
+        <v>0</v>
+      </c>
+      <c r="U336">
+        <v>0</v>
+      </c>
+      <c r="V336">
+        <v>0</v>
+      </c>
+      <c r="W336">
+        <v>0</v>
+      </c>
+      <c r="X336">
+        <v>0</v>
+      </c>
+      <c r="Y336">
         <v>3</v>
       </c>
-      <c r="Z335">
-        <v>0</v>
-      </c>
-      <c r="AA335" t="b">
+      <c r="Z336">
+        <v>0</v>
+      </c>
+      <c r="AA336" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update prep data with proper matching of leptraits by species names to get additional leptrais species data - e.g. number host plant families, voltinism
</commit_message>
<xml_diff>
--- a/data/lepidoptera_trait_data/lepidoptera_trait_data/SpeciesListForTraits.xlsx
+++ b/data/lepidoptera_trait_data/lepidoptera_trait_data/SpeciesListForTraits.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jensj\Documents\R\urban_park_community_science_project\data\lepidoptera_trait_data\lepidoptera_trait_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User.AMER-PF2237NH\Documents\R\urban_park_community_science_project\data\lepidoptera_trait_data\lepidoptera_trait_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38F63E77-3EEA-4823-94FF-C31839AD7A2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{049351F1-E5F7-4E43-830D-A92A709D50DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1620" windowWidth="21348" windowHeight="9816" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="butterflyTraits_add_missing_spe" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="953" uniqueCount="503">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="981" uniqueCount="514">
   <si>
     <t>aveWingspan</t>
   </si>
@@ -1545,6 +1545,39 @@
   </si>
   <si>
     <t>Phaeostrymon alcestis</t>
+  </si>
+  <si>
+    <t>Argynnis cybele</t>
+  </si>
+  <si>
+    <t>Mestra dorcas</t>
+  </si>
+  <si>
+    <t>Lycaena phlaeas</t>
+  </si>
+  <si>
+    <t>Argynnis callippe</t>
+  </si>
+  <si>
+    <t>Pterourus canadensis</t>
+  </si>
+  <si>
+    <t>Heraclides cresphontes</t>
+  </si>
+  <si>
+    <t>Pterourus eurymedon</t>
+  </si>
+  <si>
+    <t>Pterourus glaucus</t>
+  </si>
+  <si>
+    <t>Pterourus palamedes</t>
+  </si>
+  <si>
+    <t>Pterourus rutulus</t>
+  </si>
+  <si>
+    <t>Pterourus troilus</t>
   </si>
 </sst>
 </file>
@@ -2421,20 +2454,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AB343"/>
-  <sheetFormatPr defaultColWidth="10.83203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.83203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="19.33203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="26.83203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="19.33203125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="26.796875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.296875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="26.796875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="19.296875" style="1" customWidth="1"/>
     <col min="5" max="5" width="17" style="1" customWidth="1"/>
     <col min="6" max="6" width="20.5" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" style="1"/>
-    <col min="8" max="26" width="10.83203125" style="1" customWidth="1"/>
-    <col min="28" max="16384" width="10.83203125" style="1"/>
+    <col min="7" max="7" width="10.796875" style="1"/>
+    <col min="8" max="26" width="10.796875" style="1" customWidth="1"/>
+    <col min="28" max="16384" width="10.796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>354</v>
       </c>
@@ -2520,7 +2553,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>20</v>
       </c>
@@ -2599,11 +2632,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>21</v>
       </c>
-      <c r="B3"/>
+      <c r="B3" t="s">
+        <v>357</v>
+      </c>
       <c r="C3" t="s">
         <v>357</v>
       </c>
@@ -2676,7 +2711,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>294</v>
       </c>
@@ -2755,7 +2790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>295</v>
       </c>
@@ -2838,7 +2873,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>22</v>
       </c>
@@ -2917,7 +2952,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>23</v>
       </c>
@@ -2994,7 +3029,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -3071,7 +3106,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>309</v>
       </c>
@@ -3150,7 +3185,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>310</v>
       </c>
@@ -3229,7 +3264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>311</v>
       </c>
@@ -3308,7 +3343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -3387,7 +3422,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -3464,7 +3499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -3541,7 +3576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -3618,7 +3653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>296</v>
       </c>
@@ -3697,7 +3732,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -3774,7 +3809,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>30</v>
       </c>
@@ -3851,7 +3886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>31</v>
       </c>
@@ -3928,7 +3963,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B20" s="3" t="s">
         <v>495</v>
       </c>
@@ -3979,7 +4014,7 @@
       </c>
       <c r="AA20" s="3"/>
     </row>
-    <row r="21" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>32</v>
       </c>
@@ -4056,7 +4091,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>33</v>
       </c>
@@ -4133,7 +4168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>34</v>
       </c>
@@ -4210,7 +4245,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3"/>
       <c r="B24" s="3" t="s">
         <v>463</v>
@@ -4261,7 +4296,7 @@
       </c>
       <c r="AA24" s="3"/>
     </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>35</v>
       </c>
@@ -4338,7 +4373,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>36</v>
       </c>
@@ -4415,7 +4450,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>37</v>
       </c>
@@ -4492,7 +4527,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>38</v>
       </c>
@@ -4569,7 +4604,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>39</v>
       </c>
@@ -4646,7 +4681,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>40</v>
       </c>
@@ -4723,7 +4758,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>41</v>
       </c>
@@ -4800,7 +4835,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>42</v>
       </c>
@@ -4877,7 +4912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>43</v>
       </c>
@@ -4954,7 +4989,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>44</v>
       </c>
@@ -5031,7 +5066,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>45</v>
       </c>
@@ -5108,7 +5143,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>46</v>
       </c>
@@ -5185,7 +5220,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>47</v>
       </c>
@@ -5262,7 +5297,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>48</v>
       </c>
@@ -5339,7 +5374,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>49</v>
       </c>
@@ -5416,7 +5451,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>50</v>
       </c>
@@ -5493,7 +5528,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>51</v>
       </c>
@@ -5570,7 +5605,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>52</v>
       </c>
@@ -5649,7 +5684,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="3"/>
       <c r="B43" s="3" t="s">
         <v>467</v>
@@ -5700,7 +5735,7 @@
       </c>
       <c r="AA43" s="3"/>
     </row>
-    <row r="44" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>297</v>
       </c>
@@ -5779,7 +5814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>53</v>
       </c>
@@ -5856,7 +5891,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>54</v>
       </c>
@@ -5933,7 +5968,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>55</v>
       </c>
@@ -6010,7 +6045,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>298</v>
       </c>
@@ -6091,7 +6126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
         <v>324</v>
       </c>
@@ -6172,7 +6207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
         <v>324</v>
       </c>
@@ -6253,7 +6288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
         <v>324</v>
       </c>
@@ -6334,7 +6369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>325</v>
       </c>
@@ -6413,7 +6448,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A53" s="3"/>
       <c r="B53" s="3" t="s">
         <v>466</v>
@@ -6464,7 +6499,7 @@
       </c>
       <c r="AA53" s="3"/>
     </row>
-    <row r="54" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A54" s="3"/>
       <c r="B54" s="3" t="s">
         <v>490</v>
@@ -6515,7 +6550,7 @@
       </c>
       <c r="AA54" s="3"/>
     </row>
-    <row r="55" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>326</v>
       </c>
@@ -6594,7 +6629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>327</v>
       </c>
@@ -6673,7 +6708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>328</v>
       </c>
@@ -6752,7 +6787,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>329</v>
       </c>
@@ -6831,7 +6866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>56</v>
       </c>
@@ -6908,7 +6943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>57</v>
       </c>
@@ -6985,7 +7020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>58</v>
       </c>
@@ -7062,7 +7097,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>59</v>
       </c>
@@ -7139,7 +7174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>60</v>
       </c>
@@ -7216,7 +7251,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>61</v>
       </c>
@@ -7293,7 +7328,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>62</v>
       </c>
@@ -7370,7 +7405,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>63</v>
       </c>
@@ -7447,7 +7482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>64</v>
       </c>
@@ -7524,7 +7559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A68" s="3" t="s">
         <v>65</v>
       </c>
@@ -7603,7 +7638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>66</v>
       </c>
@@ -7680,7 +7715,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>330</v>
       </c>
@@ -7759,7 +7794,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>67</v>
       </c>
@@ -7834,7 +7869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>68</v>
       </c>
@@ -7909,7 +7944,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>69</v>
       </c>
@@ -7984,7 +8019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>70</v>
       </c>
@@ -8059,7 +8094,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>71</v>
       </c>
@@ -8138,7 +8173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>71</v>
       </c>
@@ -8219,7 +8254,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>71</v>
       </c>
@@ -8300,7 +8335,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>72</v>
       </c>
@@ -8375,7 +8410,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>73</v>
       </c>
@@ -8450,7 +8485,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>74</v>
       </c>
@@ -8525,7 +8560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A81" s="3"/>
       <c r="B81" s="3" t="s">
         <v>496</v>
@@ -8577,7 +8612,7 @@
       </c>
       <c r="AA81" s="3"/>
     </row>
-    <row r="82" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A82" s="3"/>
       <c r="B82" s="3" t="s">
         <v>469</v>
@@ -8628,7 +8663,7 @@
       </c>
       <c r="AA82" s="3"/>
     </row>
-    <row r="83" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>75</v>
       </c>
@@ -8703,7 +8738,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>76</v>
       </c>
@@ -8778,7 +8813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>77</v>
       </c>
@@ -8853,7 +8888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>78</v>
       </c>
@@ -8928,7 +8963,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>79</v>
       </c>
@@ -9003,7 +9038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>80</v>
       </c>
@@ -9078,7 +9113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>331</v>
       </c>
@@ -9157,7 +9192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A90" s="3" t="s">
         <v>81</v>
       </c>
@@ -9165,7 +9200,9 @@
         <v>470</v>
       </c>
       <c r="C90" s="3"/>
-      <c r="D90" s="3"/>
+      <c r="D90" s="3" t="s">
+        <v>81</v>
+      </c>
       <c r="E90" s="3"/>
       <c r="F90" s="3"/>
       <c r="G90" s="3">
@@ -9232,7 +9269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>82</v>
       </c>
@@ -9307,7 +9344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>83</v>
       </c>
@@ -9382,7 +9419,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>84</v>
       </c>
@@ -9457,7 +9494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>85</v>
       </c>
@@ -9532,7 +9569,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>86</v>
       </c>
@@ -9607,7 +9644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>87</v>
       </c>
@@ -9682,7 +9719,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>88</v>
       </c>
@@ -9757,7 +9794,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>89</v>
       </c>
@@ -9832,7 +9869,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>90</v>
       </c>
@@ -9840,7 +9877,9 @@
         <v>492</v>
       </c>
       <c r="C99"/>
-      <c r="D99"/>
+      <c r="D99" t="s">
+        <v>90</v>
+      </c>
       <c r="E99"/>
       <c r="F99"/>
       <c r="G99">
@@ -9907,7 +9946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>90</v>
       </c>
@@ -9982,7 +10021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>91</v>
       </c>
@@ -10057,7 +10096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A102" s="3" t="s">
         <v>91</v>
       </c>
@@ -10065,7 +10104,9 @@
         <v>488</v>
       </c>
       <c r="C102" s="3"/>
-      <c r="D102" s="3"/>
+      <c r="D102" s="3" t="s">
+        <v>91</v>
+      </c>
       <c r="E102" s="3"/>
       <c r="F102" s="3"/>
       <c r="G102" s="3">
@@ -10132,7 +10173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A103" s="3" t="s">
         <v>332</v>
       </c>
@@ -10211,7 +10252,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>333</v>
       </c>
@@ -10290,7 +10331,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>92</v>
       </c>
@@ -10298,7 +10339,9 @@
         <v>392</v>
       </c>
       <c r="C105"/>
-      <c r="D105"/>
+      <c r="D105" t="s">
+        <v>92</v>
+      </c>
       <c r="E105"/>
       <c r="F105"/>
       <c r="G105">
@@ -10365,7 +10408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>93</v>
       </c>
@@ -10440,7 +10483,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>94</v>
       </c>
@@ -10515,7 +10558,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>95</v>
       </c>
@@ -10590,7 +10633,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>96</v>
       </c>
@@ -10665,7 +10708,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>97</v>
       </c>
@@ -10740,7 +10783,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>98</v>
       </c>
@@ -10815,7 +10858,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>99</v>
       </c>
@@ -10890,7 +10933,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>100</v>
       </c>
@@ -10965,7 +11008,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>101</v>
       </c>
@@ -11040,7 +11083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>102</v>
       </c>
@@ -11115,7 +11158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>103</v>
       </c>
@@ -11190,7 +11233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>104</v>
       </c>
@@ -11265,7 +11308,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>105</v>
       </c>
@@ -11340,7 +11383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>106</v>
       </c>
@@ -11415,7 +11458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>107</v>
       </c>
@@ -11490,7 +11533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>108</v>
       </c>
@@ -11565,7 +11608,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>109</v>
       </c>
@@ -11640,7 +11683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>110</v>
       </c>
@@ -11715,7 +11758,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>111</v>
       </c>
@@ -11790,7 +11833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>112</v>
       </c>
@@ -11865,7 +11908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>113</v>
       </c>
@@ -11940,7 +11983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>114</v>
       </c>
@@ -12015,7 +12058,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>115</v>
       </c>
@@ -12090,7 +12133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>116</v>
       </c>
@@ -12165,7 +12208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>117</v>
       </c>
@@ -12240,7 +12283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>118</v>
       </c>
@@ -12315,7 +12358,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>119</v>
       </c>
@@ -12390,7 +12433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>120</v>
       </c>
@@ -12465,7 +12508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>121</v>
       </c>
@@ -12540,7 +12583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>313</v>
       </c>
@@ -12619,7 +12662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>314</v>
       </c>
@@ -12698,7 +12741,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>316</v>
       </c>
@@ -12777,7 +12820,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>122</v>
       </c>
@@ -12852,7 +12895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>123</v>
       </c>
@@ -12927,7 +12970,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>124</v>
       </c>
@@ -13002,7 +13045,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>125</v>
       </c>
@@ -13077,7 +13120,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>126</v>
       </c>
@@ -13152,7 +13195,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>127</v>
       </c>
@@ -13227,7 +13270,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>128</v>
       </c>
@@ -13302,7 +13345,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>129</v>
       </c>
@@ -13377,7 +13420,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>130</v>
       </c>
@@ -13452,7 +13495,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>131</v>
       </c>
@@ -13527,7 +13570,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>334</v>
       </c>
@@ -13606,7 +13649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>132</v>
       </c>
@@ -13681,7 +13724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>133</v>
       </c>
@@ -13756,7 +13799,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>134</v>
       </c>
@@ -13831,7 +13874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>135</v>
       </c>
@@ -13906,7 +13949,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:27" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:27" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A153" s="4"/>
       <c r="B153" s="4" t="s">
         <v>472</v>
@@ -13957,7 +14000,7 @@
       </c>
       <c r="AA153" s="4"/>
     </row>
-    <row r="154" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>136</v>
       </c>
@@ -14032,7 +14075,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>137</v>
       </c>
@@ -14107,7 +14150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A156" s="3" t="s">
         <v>138</v>
       </c>
@@ -14185,7 +14228,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>302</v>
       </c>
@@ -14262,7 +14305,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>139</v>
       </c>
@@ -14337,7 +14380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>139</v>
       </c>
@@ -14345,7 +14388,9 @@
         <v>487</v>
       </c>
       <c r="C159"/>
-      <c r="D159"/>
+      <c r="D159" t="s">
+        <v>139</v>
+      </c>
       <c r="E159"/>
       <c r="F159"/>
       <c r="G159">
@@ -14412,7 +14457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>140</v>
       </c>
@@ -14487,7 +14532,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>141</v>
       </c>
@@ -14562,7 +14607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>142</v>
       </c>
@@ -14637,7 +14682,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:27" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:27" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>143</v>
       </c>
@@ -14712,7 +14757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>144</v>
       </c>
@@ -14787,7 +14832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>145</v>
       </c>
@@ -14864,7 +14909,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="166" spans="1:27" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:27" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A166" s="4" t="s">
         <v>146</v>
       </c>
@@ -14943,7 +14988,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167" spans="1:27" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:27" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A167" s="4" t="s">
         <v>146</v>
       </c>
@@ -15022,7 +15067,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>147</v>
       </c>
@@ -15097,7 +15142,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>148</v>
       </c>
@@ -15172,7 +15217,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>149</v>
       </c>
@@ -15249,7 +15294,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>150</v>
       </c>
@@ -15324,7 +15369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>151</v>
       </c>
@@ -15399,7 +15444,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>152</v>
       </c>
@@ -15476,7 +15521,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>153</v>
       </c>
@@ -15551,7 +15596,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="175" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>303</v>
       </c>
@@ -15630,7 +15675,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>304</v>
       </c>
@@ -15709,7 +15754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>305</v>
       </c>
@@ -15788,7 +15833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>306</v>
       </c>
@@ -15867,7 +15912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>154</v>
       </c>
@@ -15944,7 +15989,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="180" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>155</v>
       </c>
@@ -16019,7 +16064,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="181" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>156</v>
       </c>
@@ -16094,7 +16139,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:27" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:27" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A182" s="4" t="s">
         <v>156</v>
       </c>
@@ -16102,7 +16147,9 @@
         <v>482</v>
       </c>
       <c r="C182" s="4"/>
-      <c r="D182" s="4"/>
+      <c r="D182" s="4" t="s">
+        <v>156</v>
+      </c>
       <c r="E182" s="4"/>
       <c r="F182" s="4"/>
       <c r="G182" s="4">
@@ -16167,7 +16214,7 @@
       </c>
       <c r="AA182" s="4"/>
     </row>
-    <row r="183" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>157</v>
       </c>
@@ -16242,7 +16289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>158</v>
       </c>
@@ -16317,7 +16364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>159</v>
       </c>
@@ -16392,7 +16439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>160</v>
       </c>
@@ -16467,7 +16514,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>308</v>
       </c>
@@ -16546,7 +16593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>161</v>
       </c>
@@ -16621,7 +16668,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>162</v>
       </c>
@@ -16696,7 +16743,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>163</v>
       </c>
@@ -16771,7 +16818,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="191" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>164</v>
       </c>
@@ -16846,7 +16893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>165</v>
       </c>
@@ -16856,7 +16903,9 @@
       <c r="C192" t="s">
         <v>412</v>
       </c>
-      <c r="D192"/>
+      <c r="D192" t="s">
+        <v>165</v>
+      </c>
       <c r="E192"/>
       <c r="F192"/>
       <c r="G192">
@@ -16923,7 +16972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>166</v>
       </c>
@@ -16998,7 +17047,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>167</v>
       </c>
@@ -17073,7 +17122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>168</v>
       </c>
@@ -17081,7 +17130,9 @@
         <v>415</v>
       </c>
       <c r="C195"/>
-      <c r="D195"/>
+      <c r="D195" t="s">
+        <v>505</v>
+      </c>
       <c r="E195"/>
       <c r="F195"/>
       <c r="G195">
@@ -17148,7 +17199,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="196" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>169</v>
       </c>
@@ -17223,7 +17274,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="197" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>335</v>
       </c>
@@ -17302,7 +17353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>336</v>
       </c>
@@ -17381,7 +17432,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>170</v>
       </c>
@@ -17456,7 +17507,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>171</v>
       </c>
@@ -17464,7 +17515,9 @@
         <v>171</v>
       </c>
       <c r="C200"/>
-      <c r="D200"/>
+      <c r="D200" t="s">
+        <v>504</v>
+      </c>
       <c r="E200"/>
       <c r="F200"/>
       <c r="G200" t="s">
@@ -17531,7 +17584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>172</v>
       </c>
@@ -17606,7 +17659,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>173</v>
       </c>
@@ -17681,7 +17734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>174</v>
       </c>
@@ -17756,7 +17809,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="204" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>175</v>
       </c>
@@ -17831,7 +17884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>176</v>
       </c>
@@ -17906,7 +17959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>177</v>
       </c>
@@ -17981,7 +18034,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="207" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>178</v>
       </c>
@@ -18056,7 +18109,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>179</v>
       </c>
@@ -18131,7 +18184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>180</v>
       </c>
@@ -18206,7 +18259,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="210" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>181</v>
       </c>
@@ -18281,7 +18334,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="211" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>337</v>
       </c>
@@ -18360,7 +18413,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="212" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>183</v>
       </c>
@@ -18435,7 +18488,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A213" s="3"/>
       <c r="B213" s="3" t="s">
         <v>474</v>
@@ -18486,7 +18539,7 @@
       </c>
       <c r="AA213" s="3"/>
     </row>
-    <row r="214" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>184</v>
       </c>
@@ -18561,7 +18614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>185</v>
       </c>
@@ -18636,7 +18689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>186</v>
       </c>
@@ -18711,7 +18764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>187</v>
       </c>
@@ -18786,7 +18839,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>188</v>
       </c>
@@ -18861,7 +18914,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>189</v>
       </c>
@@ -18936,7 +18989,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>190</v>
       </c>
@@ -19011,7 +19064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A221" s="3"/>
       <c r="B221" s="3" t="s">
         <v>475</v>
@@ -19062,7 +19115,7 @@
       </c>
       <c r="AA221" s="3"/>
     </row>
-    <row r="222" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>191</v>
       </c>
@@ -19137,7 +19190,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="223" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>192</v>
       </c>
@@ -19212,7 +19265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>193</v>
       </c>
@@ -19287,7 +19340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>194</v>
       </c>
@@ -19295,7 +19348,9 @@
         <v>194</v>
       </c>
       <c r="C225"/>
-      <c r="D225"/>
+      <c r="D225" t="s">
+        <v>507</v>
+      </c>
       <c r="E225"/>
       <c r="F225"/>
       <c r="G225">
@@ -19362,7 +19417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>195</v>
       </c>
@@ -19370,7 +19425,9 @@
         <v>195</v>
       </c>
       <c r="C226"/>
-      <c r="D226"/>
+      <c r="D226" t="s">
+        <v>508</v>
+      </c>
       <c r="E226"/>
       <c r="F226"/>
       <c r="G226" t="s">
@@ -19437,7 +19494,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="227" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>196</v>
       </c>
@@ -19445,7 +19502,9 @@
         <v>196</v>
       </c>
       <c r="C227"/>
-      <c r="D227"/>
+      <c r="D227" t="s">
+        <v>509</v>
+      </c>
       <c r="E227"/>
       <c r="F227"/>
       <c r="G227">
@@ -19512,7 +19571,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>197</v>
       </c>
@@ -19520,7 +19579,9 @@
         <v>197</v>
       </c>
       <c r="C228"/>
-      <c r="D228"/>
+      <c r="D228" t="s">
+        <v>510</v>
+      </c>
       <c r="E228"/>
       <c r="F228"/>
       <c r="G228">
@@ -19587,7 +19648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>198</v>
       </c>
@@ -19662,7 +19723,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="230" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>199</v>
       </c>
@@ -19737,7 +19798,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="231" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>200</v>
       </c>
@@ -19812,7 +19873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="232" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>201</v>
       </c>
@@ -19820,7 +19881,9 @@
         <v>201</v>
       </c>
       <c r="C232"/>
-      <c r="D232"/>
+      <c r="D232" t="s">
+        <v>511</v>
+      </c>
       <c r="E232"/>
       <c r="F232"/>
       <c r="G232">
@@ -19887,7 +19950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="233" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A233" s="3"/>
       <c r="B233" s="3" t="s">
         <v>476</v>
@@ -19938,7 +20001,7 @@
       </c>
       <c r="AA233" s="3"/>
     </row>
-    <row r="234" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>202</v>
       </c>
@@ -19946,7 +20009,9 @@
         <v>202</v>
       </c>
       <c r="C234"/>
-      <c r="D234"/>
+      <c r="D234" t="s">
+        <v>508</v>
+      </c>
       <c r="E234"/>
       <c r="F234"/>
       <c r="G234">
@@ -20013,7 +20078,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="235" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>203</v>
       </c>
@@ -20021,7 +20086,9 @@
         <v>203</v>
       </c>
       <c r="C235"/>
-      <c r="D235"/>
+      <c r="D235" t="s">
+        <v>512</v>
+      </c>
       <c r="E235"/>
       <c r="F235"/>
       <c r="G235" s="3">
@@ -20091,7 +20158,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="236" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>204</v>
       </c>
@@ -20099,7 +20166,9 @@
         <v>204</v>
       </c>
       <c r="C236"/>
-      <c r="D236"/>
+      <c r="D236" t="s">
+        <v>513</v>
+      </c>
       <c r="E236"/>
       <c r="F236"/>
       <c r="G236">
@@ -20166,7 +20235,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="237" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>205</v>
       </c>
@@ -20241,7 +20310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="238" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>206</v>
       </c>
@@ -20316,7 +20385,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="239" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>207</v>
       </c>
@@ -20391,7 +20460,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="240" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>208</v>
       </c>
@@ -20466,7 +20535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="241" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A241" s="3"/>
       <c r="B241" s="3" t="s">
         <v>502</v>
@@ -20518,7 +20587,7 @@
       </c>
       <c r="AA241" s="3"/>
     </row>
-    <row r="242" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A242" s="3"/>
       <c r="B242" s="3" t="s">
         <v>477</v>
@@ -20569,7 +20638,7 @@
       </c>
       <c r="AA242" s="3"/>
     </row>
-    <row r="243" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>318</v>
       </c>
@@ -20648,7 +20717,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="244" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>209</v>
       </c>
@@ -20723,7 +20792,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="245" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>210</v>
       </c>
@@ -20798,7 +20867,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="246" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>211</v>
       </c>
@@ -20806,7 +20875,9 @@
         <v>491</v>
       </c>
       <c r="C246"/>
-      <c r="D246"/>
+      <c r="D246" t="s">
+        <v>211</v>
+      </c>
       <c r="E246"/>
       <c r="F246"/>
       <c r="G246">
@@ -20873,7 +20944,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="247" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A247" s="3" t="s">
         <v>211</v>
       </c>
@@ -20948,7 +21019,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="248" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>212</v>
       </c>
@@ -21023,7 +21094,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="249" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>213</v>
       </c>
@@ -21098,7 +21169,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="250" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>214</v>
       </c>
@@ -21173,7 +21244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="251" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>319</v>
       </c>
@@ -21252,7 +21323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="252" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A252" s="3" t="s">
         <v>300</v>
       </c>
@@ -21331,7 +21402,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="253" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>300</v>
       </c>
@@ -21410,7 +21481,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="254" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>215</v>
       </c>
@@ -21485,7 +21556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="255" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>216</v>
       </c>
@@ -21560,7 +21631,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="256" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>217</v>
       </c>
@@ -21637,7 +21708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="257" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>218</v>
       </c>
@@ -21712,7 +21783,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="258" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
         <v>219</v>
       </c>
@@ -21787,7 +21858,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="259" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>220</v>
       </c>
@@ -21862,7 +21933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="260" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>221</v>
       </c>
@@ -21937,7 +22008,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="261" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>222</v>
       </c>
@@ -22012,7 +22083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="262" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>223</v>
       </c>
@@ -22089,7 +22160,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="263" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>224</v>
       </c>
@@ -22164,7 +22235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="264" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>225</v>
       </c>
@@ -22241,7 +22312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="265" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>353</v>
       </c>
@@ -22320,7 +22391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="266" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
         <v>226</v>
       </c>
@@ -22395,7 +22466,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="267" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>227</v>
       </c>
@@ -22472,7 +22543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="268" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
         <v>307</v>
       </c>
@@ -22551,7 +22622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="269" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
         <v>228</v>
       </c>
@@ -22628,7 +22699,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="270" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A270" t="s">
         <v>229</v>
       </c>
@@ -22636,7 +22707,9 @@
         <v>429</v>
       </c>
       <c r="C270"/>
-      <c r="D270"/>
+      <c r="D270" t="s">
+        <v>229</v>
+      </c>
       <c r="E270"/>
       <c r="F270"/>
       <c r="G270">
@@ -22703,7 +22776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="271" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
         <v>230</v>
       </c>
@@ -22778,7 +22851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="272" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
         <v>317</v>
       </c>
@@ -22857,7 +22930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="273" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
         <v>231</v>
       </c>
@@ -22932,7 +23005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="274" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
         <v>232</v>
       </c>
@@ -23007,7 +23080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="275" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
         <v>233</v>
       </c>
@@ -23015,7 +23088,9 @@
         <v>432</v>
       </c>
       <c r="C275"/>
-      <c r="D275"/>
+      <c r="D275" t="s">
+        <v>233</v>
+      </c>
       <c r="E275"/>
       <c r="F275"/>
       <c r="G275">
@@ -23082,7 +23157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="276" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
         <v>234</v>
       </c>
@@ -23157,7 +23232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="277" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
         <v>235</v>
       </c>
@@ -23232,7 +23307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="278" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
         <v>236</v>
       </c>
@@ -23310,7 +23385,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="279" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>237</v>
       </c>
@@ -23385,7 +23460,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="280" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
         <v>238</v>
       </c>
@@ -23460,7 +23535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="281" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
         <v>239</v>
       </c>
@@ -23535,7 +23610,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="282" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
         <v>240</v>
       </c>
@@ -23610,7 +23685,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="283" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
         <v>241</v>
       </c>
@@ -23685,7 +23760,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="284" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
         <v>242</v>
       </c>
@@ -23760,7 +23835,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="285" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
         <v>243</v>
       </c>
@@ -23835,7 +23910,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="286" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>244</v>
       </c>
@@ -23910,7 +23985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="287" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
         <v>245</v>
       </c>
@@ -23985,7 +24060,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="288" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
         <v>246</v>
       </c>
@@ -24060,7 +24135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="289" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
         <v>247</v>
       </c>
@@ -24135,14 +24210,16 @@
         <v>1</v>
       </c>
     </row>
-    <row r="290" spans="1:27" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:27" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A290" s="4" t="s">
         <v>248</v>
       </c>
       <c r="B290" s="4" t="s">
         <v>434</v>
       </c>
-      <c r="D290" s="4"/>
+      <c r="D290" s="4" t="s">
+        <v>248</v>
+      </c>
       <c r="E290" s="4"/>
       <c r="F290" s="4"/>
       <c r="G290" s="4">
@@ -24209,7 +24286,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="291" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
         <v>249</v>
       </c>
@@ -24284,7 +24361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="292" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A292" t="s">
         <v>250</v>
       </c>
@@ -24359,7 +24436,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="293" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
         <v>251</v>
       </c>
@@ -24434,7 +24511,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="294" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A294" t="s">
         <v>252</v>
       </c>
@@ -24509,7 +24586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="295" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A295" t="s">
         <v>253</v>
       </c>
@@ -24584,7 +24661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="296" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
         <v>254</v>
       </c>
@@ -24659,7 +24736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="297" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A297" t="s">
         <v>255</v>
       </c>
@@ -24667,7 +24744,9 @@
         <v>436</v>
       </c>
       <c r="C297"/>
-      <c r="D297"/>
+      <c r="D297" t="s">
+        <v>255</v>
+      </c>
       <c r="E297"/>
       <c r="F297"/>
       <c r="G297">
@@ -24734,7 +24813,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="298" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
         <v>256</v>
       </c>
@@ -24744,7 +24823,9 @@
       <c r="C298" t="s">
         <v>437</v>
       </c>
-      <c r="D298"/>
+      <c r="D298" t="s">
+        <v>255</v>
+      </c>
       <c r="E298"/>
       <c r="F298"/>
       <c r="G298">
@@ -24811,7 +24892,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="299" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
         <v>257</v>
       </c>
@@ -24886,7 +24967,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="300" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
         <v>258</v>
       </c>
@@ -24963,7 +25044,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="301" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>259</v>
       </c>
@@ -25038,7 +25119,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="302" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>260</v>
       </c>
@@ -25113,7 +25194,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="303" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>312</v>
       </c>
@@ -25192,7 +25273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="304" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>261</v>
       </c>
@@ -25267,7 +25348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="305" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>262</v>
       </c>
@@ -25342,7 +25423,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="306" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>263</v>
       </c>
@@ -25419,7 +25500,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="307" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>264</v>
       </c>
@@ -25494,7 +25575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="308" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
         <v>265</v>
       </c>
@@ -25569,7 +25650,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="309" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
         <v>266</v>
       </c>
@@ -25644,7 +25725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="310" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A310" t="s">
         <v>339</v>
       </c>
@@ -25721,7 +25802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="311" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A311" t="s">
         <v>267</v>
       </c>
@@ -25796,7 +25877,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="312" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A312" t="s">
         <v>320</v>
       </c>
@@ -25875,7 +25956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="313" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A313" t="s">
         <v>301</v>
       </c>
@@ -25954,7 +26035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="314" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A314" t="s">
         <v>268</v>
       </c>
@@ -26029,7 +26110,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="315" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A315" t="s">
         <v>269</v>
       </c>
@@ -26104,7 +26185,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="316" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A316" t="s">
         <v>270</v>
       </c>
@@ -26112,7 +26193,9 @@
         <v>445</v>
       </c>
       <c r="C316"/>
-      <c r="D316"/>
+      <c r="D316" t="s">
+        <v>506</v>
+      </c>
       <c r="E316"/>
       <c r="F316"/>
       <c r="G316">
@@ -26179,7 +26262,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="317" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A317" t="s">
         <v>271</v>
       </c>
@@ -26187,7 +26270,9 @@
         <v>446</v>
       </c>
       <c r="C317"/>
-      <c r="D317"/>
+      <c r="D317" t="s">
+        <v>503</v>
+      </c>
       <c r="E317"/>
       <c r="F317"/>
       <c r="G317">
@@ -26254,7 +26339,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="318" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A318" t="s">
         <v>272</v>
       </c>
@@ -26329,7 +26414,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="319" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A319" t="s">
         <v>273</v>
       </c>
@@ -26404,7 +26489,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="320" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A320" t="s">
         <v>274</v>
       </c>
@@ -26479,7 +26564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="321" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A321" t="s">
         <v>275</v>
       </c>
@@ -26554,7 +26639,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="322" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A322" t="s">
         <v>276</v>
       </c>
@@ -26629,7 +26714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="323" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A323" t="s">
         <v>277</v>
       </c>
@@ -26704,7 +26789,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="324" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A324" t="s">
         <v>278</v>
       </c>
@@ -26779,7 +26864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="325" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A325" t="s">
         <v>279</v>
       </c>
@@ -26854,7 +26939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="326" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A326" t="s">
         <v>280</v>
       </c>
@@ -26929,7 +27014,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="327" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A327" s="3"/>
       <c r="B327" s="3" t="s">
         <v>479</v>
@@ -26980,7 +27065,7 @@
       </c>
       <c r="AA327" s="3"/>
     </row>
-    <row r="328" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A328" t="s">
         <v>281</v>
       </c>
@@ -27055,7 +27140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="329" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A329" t="s">
         <v>282</v>
       </c>
@@ -27130,7 +27215,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="330" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A330" t="s">
         <v>283</v>
       </c>
@@ -27205,7 +27290,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="331" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A331" t="s">
         <v>340</v>
       </c>
@@ -27284,7 +27369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="332" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A332" t="s">
         <v>284</v>
       </c>
@@ -27359,7 +27444,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="333" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A333" t="s">
         <v>285</v>
       </c>
@@ -27434,7 +27519,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="334" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A334" t="s">
         <v>286</v>
       </c>
@@ -27509,7 +27594,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="335" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A335" t="s">
         <v>287</v>
       </c>
@@ -27584,7 +27669,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="336" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A336" t="s">
         <v>288</v>
       </c>
@@ -27659,7 +27744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="337" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:27" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A337" s="3" t="s">
         <v>299</v>
       </c>
@@ -27738,7 +27823,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="338" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A338" t="s">
         <v>289</v>
       </c>
@@ -27813,7 +27898,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="339" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A339" t="s">
         <v>290</v>
       </c>
@@ -27888,7 +27973,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="340" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A340" t="s">
         <v>291</v>
       </c>
@@ -27963,7 +28048,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="341" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A341" t="s">
         <v>292</v>
       </c>
@@ -27973,7 +28058,9 @@
       <c r="C341" t="s">
         <v>451</v>
       </c>
-      <c r="D341"/>
+      <c r="D341" t="s">
+        <v>292</v>
+      </c>
       <c r="E341"/>
       <c r="F341"/>
       <c r="G341">
@@ -28040,7 +28127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="342" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A342" t="s">
         <v>292</v>
       </c>
@@ -28050,7 +28137,9 @@
       <c r="C342" t="s">
         <v>451</v>
       </c>
-      <c r="D342"/>
+      <c r="D342" t="s">
+        <v>292</v>
+      </c>
       <c r="E342"/>
       <c r="F342"/>
       <c r="G342">
@@ -28117,7 +28206,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="343" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A343" t="s">
         <v>293</v>
       </c>

</xml_diff>